<commit_message>
Tweaked additional models' scaling and orientation
</commit_message>
<xml_diff>
--- a/SpectrobesSFM checklist.xlsx
+++ b/SpectrobesSFM checklist.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="526">
   <si>
     <t>name</t>
   </si>
@@ -2124,6 +2124,15 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2154,15 +2163,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2416,22 +2416,22 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="12.75">
-      <c r="A2" s="56" t="s">
+      <c r="A2" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="57"/>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="58"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="61"/>
     </row>
     <row r="3" spans="1:6" ht="13.5" thickBot="1">
-      <c r="A3" s="59"/>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="61"/>
+      <c r="A3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="64"/>
     </row>
     <row r="4" spans="1:6" ht="12.75">
       <c r="A4" s="4" t="s">
@@ -2632,22 +2632,22 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="12.75">
-      <c r="A15" s="56" t="s">
+      <c r="A15" s="59" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="57"/>
-      <c r="C15" s="57"/>
-      <c r="D15" s="57"/>
-      <c r="E15" s="57"/>
-      <c r="F15" s="58"/>
+      <c r="B15" s="60"/>
+      <c r="C15" s="60"/>
+      <c r="D15" s="60"/>
+      <c r="E15" s="60"/>
+      <c r="F15" s="61"/>
     </row>
     <row r="16" spans="1:6" ht="13.5" thickBot="1">
-      <c r="A16" s="59"/>
-      <c r="B16" s="60"/>
-      <c r="C16" s="60"/>
-      <c r="D16" s="60"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="61"/>
+      <c r="A16" s="62"/>
+      <c r="B16" s="63"/>
+      <c r="C16" s="63"/>
+      <c r="D16" s="63"/>
+      <c r="E16" s="63"/>
+      <c r="F16" s="64"/>
     </row>
     <row r="17" spans="1:6" ht="12.75">
       <c r="A17" s="19" t="s">
@@ -2656,7 +2656,7 @@
       <c r="B17" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="C17" s="73" t="s">
+      <c r="C17" s="56" t="s">
         <v>423</v>
       </c>
       <c r="D17" s="49" t="s">
@@ -2988,22 +2988,22 @@
       <c r="F46" s="9"/>
     </row>
     <row r="47" spans="1:6" ht="12.75">
-      <c r="A47" s="62" t="s">
+      <c r="A47" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="B47" s="57"/>
-      <c r="C47" s="57"/>
-      <c r="D47" s="57"/>
-      <c r="E47" s="57"/>
-      <c r="F47" s="58"/>
+      <c r="B47" s="60"/>
+      <c r="C47" s="60"/>
+      <c r="D47" s="60"/>
+      <c r="E47" s="60"/>
+      <c r="F47" s="61"/>
     </row>
     <row r="48" spans="1:6" ht="13.5" thickBot="1">
-      <c r="A48" s="59"/>
-      <c r="B48" s="60"/>
-      <c r="C48" s="60"/>
-      <c r="D48" s="60"/>
-      <c r="E48" s="60"/>
-      <c r="F48" s="61"/>
+      <c r="A48" s="62"/>
+      <c r="B48" s="63"/>
+      <c r="C48" s="63"/>
+      <c r="D48" s="63"/>
+      <c r="E48" s="63"/>
+      <c r="F48" s="64"/>
     </row>
     <row r="49" spans="1:6" ht="12.75">
       <c r="A49" s="11" t="s">
@@ -3012,13 +3012,13 @@
       <c r="B49" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="C49" s="73" t="s">
+      <c r="C49" s="56" t="s">
         <v>423</v>
       </c>
-      <c r="D49" s="74" t="s">
+      <c r="D49" s="57" t="s">
         <v>423</v>
       </c>
-      <c r="E49" s="75"/>
+      <c r="E49" s="58"/>
       <c r="F49" s="50" t="s">
         <v>423</v>
       </c>
@@ -3174,10 +3174,16 @@
       <c r="B58" s="25" t="s">
         <v>173</v>
       </c>
-      <c r="C58" s="13"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="8"/>
-      <c r="F58" s="9"/>
+      <c r="C58" s="47" t="s">
+        <v>423</v>
+      </c>
+      <c r="D58" s="48" t="s">
+        <v>423</v>
+      </c>
+      <c r="E58" s="45"/>
+      <c r="F58" s="46" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="59" spans="1:6" ht="12.75">
       <c r="A59" s="12" t="s">
@@ -3186,10 +3192,16 @@
       <c r="B59" s="25" t="s">
         <v>174</v>
       </c>
-      <c r="C59" s="13"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="8"/>
-      <c r="F59" s="9"/>
+      <c r="C59" s="47" t="s">
+        <v>423</v>
+      </c>
+      <c r="D59" s="48" t="s">
+        <v>423</v>
+      </c>
+      <c r="E59" s="45"/>
+      <c r="F59" s="46" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="60" spans="1:6" ht="12.75">
       <c r="A60" s="12" t="s">
@@ -3198,10 +3210,16 @@
       <c r="B60" s="25" t="s">
         <v>175</v>
       </c>
-      <c r="C60" s="13"/>
-      <c r="D60" s="14"/>
-      <c r="E60" s="8"/>
-      <c r="F60" s="9"/>
+      <c r="C60" s="47" t="s">
+        <v>423</v>
+      </c>
+      <c r="D60" s="48" t="s">
+        <v>423</v>
+      </c>
+      <c r="E60" s="45"/>
+      <c r="F60" s="46" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="61" spans="1:6" ht="12.75">
       <c r="A61" s="12" t="s">
@@ -3210,10 +3228,16 @@
       <c r="B61" s="25" t="s">
         <v>176</v>
       </c>
-      <c r="C61" s="13"/>
-      <c r="D61" s="14"/>
-      <c r="E61" s="8"/>
-      <c r="F61" s="9"/>
+      <c r="C61" s="47" t="s">
+        <v>423</v>
+      </c>
+      <c r="D61" s="48" t="s">
+        <v>423</v>
+      </c>
+      <c r="E61" s="45"/>
+      <c r="F61" s="46" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="62" spans="1:6" ht="12.75">
       <c r="A62" s="12" t="s">
@@ -3222,10 +3246,16 @@
       <c r="B62" s="25" t="s">
         <v>177</v>
       </c>
-      <c r="C62" s="13"/>
-      <c r="D62" s="14"/>
-      <c r="E62" s="8"/>
-      <c r="F62" s="9"/>
+      <c r="C62" s="47" t="s">
+        <v>423</v>
+      </c>
+      <c r="D62" s="48" t="s">
+        <v>423</v>
+      </c>
+      <c r="E62" s="45"/>
+      <c r="F62" s="46" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="63" spans="1:6" ht="12.75">
       <c r="A63" s="12" t="s">
@@ -3234,10 +3264,16 @@
       <c r="B63" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="C63" s="13"/>
-      <c r="D63" s="14"/>
-      <c r="E63" s="8"/>
-      <c r="F63" s="9"/>
+      <c r="C63" s="47" t="s">
+        <v>423</v>
+      </c>
+      <c r="D63" s="48" t="s">
+        <v>423</v>
+      </c>
+      <c r="E63" s="45"/>
+      <c r="F63" s="46" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="64" spans="1:6" ht="12.75">
       <c r="A64" s="12" t="s">
@@ -3246,10 +3282,16 @@
       <c r="B64" s="25" t="s">
         <v>179</v>
       </c>
-      <c r="C64" s="13"/>
-      <c r="D64" s="14"/>
-      <c r="E64" s="8"/>
-      <c r="F64" s="9"/>
+      <c r="C64" s="47" t="s">
+        <v>423</v>
+      </c>
+      <c r="D64" s="48" t="s">
+        <v>423</v>
+      </c>
+      <c r="E64" s="45"/>
+      <c r="F64" s="46" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="65" spans="1:6" ht="12.75">
       <c r="A65" s="12" t="s">
@@ -4140,22 +4182,22 @@
       <c r="F138" s="9"/>
     </row>
     <row r="139" spans="1:6" ht="12.75">
-      <c r="A139" s="63" t="s">
+      <c r="A139" s="66" t="s">
         <v>119</v>
       </c>
-      <c r="B139" s="64"/>
-      <c r="C139" s="64"/>
-      <c r="D139" s="64"/>
-      <c r="E139" s="64"/>
-      <c r="F139" s="65"/>
+      <c r="B139" s="67"/>
+      <c r="C139" s="67"/>
+      <c r="D139" s="67"/>
+      <c r="E139" s="67"/>
+      <c r="F139" s="68"/>
     </row>
     <row r="140" spans="1:6" ht="13.5" thickBot="1">
-      <c r="A140" s="66"/>
-      <c r="B140" s="67"/>
-      <c r="C140" s="67"/>
-      <c r="D140" s="67"/>
-      <c r="E140" s="67"/>
-      <c r="F140" s="68"/>
+      <c r="A140" s="69"/>
+      <c r="B140" s="70"/>
+      <c r="C140" s="70"/>
+      <c r="D140" s="70"/>
+      <c r="E140" s="70"/>
+      <c r="F140" s="71"/>
     </row>
     <row r="141" spans="1:6" ht="12.75">
       <c r="A141" s="33" t="s">
@@ -5178,23 +5220,23 @@
       <c r="F225" s="32"/>
     </row>
     <row r="226" spans="1:7" ht="12.75">
-      <c r="A226" s="69" t="s">
+      <c r="A226" s="72" t="s">
         <v>425</v>
       </c>
-      <c r="B226" s="69"/>
-      <c r="C226" s="69"/>
-      <c r="D226" s="69"/>
-      <c r="E226" s="69"/>
-      <c r="F226" s="70"/>
+      <c r="B226" s="72"/>
+      <c r="C226" s="72"/>
+      <c r="D226" s="72"/>
+      <c r="E226" s="72"/>
+      <c r="F226" s="73"/>
       <c r="G226" s="51"/>
     </row>
     <row r="227" spans="1:7" ht="13.5" thickBot="1">
-      <c r="A227" s="71"/>
-      <c r="B227" s="71"/>
-      <c r="C227" s="71"/>
-      <c r="D227" s="71"/>
-      <c r="E227" s="71"/>
-      <c r="F227" s="72"/>
+      <c r="A227" s="74"/>
+      <c r="B227" s="74"/>
+      <c r="C227" s="74"/>
+      <c r="D227" s="74"/>
+      <c r="E227" s="74"/>
+      <c r="F227" s="75"/>
       <c r="G227" s="51"/>
     </row>
     <row r="228" spans="1:7" ht="12.75">

</xml_diff>

<commit_message>
adjusted more models (orientation, scale) and removed textures
</commit_message>
<xml_diff>
--- a/SpectrobesSFM checklist.xlsx
+++ b/SpectrobesSFM checklist.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="526">
   <si>
     <t>name</t>
   </si>
@@ -3300,10 +3300,16 @@
       <c r="B65" s="25" t="s">
         <v>180</v>
       </c>
-      <c r="C65" s="13"/>
-      <c r="D65" s="14"/>
-      <c r="E65" s="8"/>
-      <c r="F65" s="9"/>
+      <c r="C65" s="47" t="s">
+        <v>423</v>
+      </c>
+      <c r="D65" s="48" t="s">
+        <v>423</v>
+      </c>
+      <c r="E65" s="45"/>
+      <c r="F65" s="46" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="66" spans="1:6" ht="12.75">
       <c r="A66" s="12" t="s">
@@ -3312,10 +3318,16 @@
       <c r="B66" s="25" t="s">
         <v>181</v>
       </c>
-      <c r="C66" s="13"/>
-      <c r="D66" s="14"/>
-      <c r="E66" s="8"/>
-      <c r="F66" s="9"/>
+      <c r="C66" s="47" t="s">
+        <v>423</v>
+      </c>
+      <c r="D66" s="48" t="s">
+        <v>423</v>
+      </c>
+      <c r="E66" s="45"/>
+      <c r="F66" s="46" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="67" spans="1:6" ht="12.75">
       <c r="A67" s="12" t="s">
@@ -3324,10 +3336,16 @@
       <c r="B67" s="25" t="s">
         <v>182</v>
       </c>
-      <c r="C67" s="13"/>
-      <c r="D67" s="14"/>
-      <c r="E67" s="8"/>
-      <c r="F67" s="9"/>
+      <c r="C67" s="47" t="s">
+        <v>423</v>
+      </c>
+      <c r="D67" s="48" t="s">
+        <v>423</v>
+      </c>
+      <c r="E67" s="45"/>
+      <c r="F67" s="46" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="68" spans="1:6" ht="12.75">
       <c r="A68" s="12" t="s">
@@ -3336,10 +3354,16 @@
       <c r="B68" s="25" t="s">
         <v>183</v>
       </c>
-      <c r="C68" s="13"/>
-      <c r="D68" s="14"/>
-      <c r="E68" s="8"/>
-      <c r="F68" s="9"/>
+      <c r="C68" s="47" t="s">
+        <v>423</v>
+      </c>
+      <c r="D68" s="48" t="s">
+        <v>423</v>
+      </c>
+      <c r="E68" s="45"/>
+      <c r="F68" s="46" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="69" spans="1:6" ht="12.75">
       <c r="A69" s="12" t="s">
@@ -3348,10 +3372,16 @@
       <c r="B69" s="25" t="s">
         <v>184</v>
       </c>
-      <c r="C69" s="13"/>
-      <c r="D69" s="14"/>
-      <c r="E69" s="8"/>
-      <c r="F69" s="9"/>
+      <c r="C69" s="47" t="s">
+        <v>423</v>
+      </c>
+      <c r="D69" s="48" t="s">
+        <v>423</v>
+      </c>
+      <c r="E69" s="45"/>
+      <c r="F69" s="46" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="70" spans="1:6" ht="12.75">
       <c r="A70" s="12" t="s">

</xml_diff>